<commit_message>
feat(tables): synchronize sample efficiency, pairwise anchor, token budget tables and compendium pdf
- Recompute sample efficiency study across all 14 datasets and update sample_efficiency_macro.tex, sample_efficiency_macro_m3.tex, and sample_efficiency_macro_mqt.tex
- Re-run pairwise anchor mining script to update pairwise_anchor_summary.tex
- Recompute token budget experiment across 9 benchmarks and update token_budget/ LaTeX tables and Pareto figures
- Recompile all_tables_compendium.pdf incorporating all freshly generated LaTeX tables
- Verify 100% test passage (163/163 passed) and pre-commit hook compliance
</commit_message>
<xml_diff>
--- a/sheets/sample_efficiency_results.xlsx
+++ b/sheets/sample_efficiency_results.xlsx
@@ -538,25 +538,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>40.4697</v>
+        <v>41.2313</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>40.4332</v>
+        <v>41.2396</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.3973</v>
+        <v>0.4023</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -582,25 +582,25 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>22.9821</v>
+        <v>23.1856</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1297</v>
+        <v>0.1537</v>
       </c>
       <c r="F3" t="n">
-        <v>22.2103</v>
+        <v>22.4249</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1394</v>
+        <v>0.1778</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2222</v>
+        <v>0.2245</v>
       </c>
       <c r="K3" t="n">
         <v>0.0005</v>
@@ -626,28 +626,28 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6.9734</v>
+        <v>6.9268</v>
       </c>
       <c r="E4" t="n">
-        <v>0.383</v>
+        <v>0.495</v>
       </c>
       <c r="F4" t="n">
-        <v>5.5238</v>
+        <v>5.6404</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5678</v>
+        <v>0.7389</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6845</v>
+        <v>0.6937</v>
       </c>
       <c r="I4" t="n">
         <v>0.0116</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1395</v>
+        <v>0.1413</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0013</v>
+        <v>0.0014</v>
       </c>
       <c r="L4" t="n">
         <v>50</v>
@@ -670,28 +670,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7.6162</v>
+        <v>7.5806</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4988</v>
+        <v>0.5078</v>
       </c>
       <c r="F5" t="n">
-        <v>6.7854</v>
+        <v>6.7904</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7455000000000001</v>
+        <v>0.5952</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6639</v>
+        <v>0.6737</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0145</v>
+        <v>0.0138</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1438</v>
+        <v>0.1456</v>
       </c>
       <c r="K5" t="n">
-        <v>0.0005</v>
+        <v>0.001</v>
       </c>
       <c r="L5" t="n">
         <v>50</v>
@@ -714,28 +714,28 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7.9629</v>
+        <v>7.9243</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4909</v>
+        <v>0.4453</v>
       </c>
       <c r="F6" t="n">
-        <v>6.8734</v>
+        <v>6.9042</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8177</v>
+        <v>0.8883</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6781</v>
+        <v>0.6874</v>
       </c>
       <c r="I6" t="n">
         <v>0.011</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1428</v>
+        <v>0.1445</v>
       </c>
       <c r="K6" t="n">
-        <v>0.003</v>
+        <v>0.0027</v>
       </c>
       <c r="L6" t="n">
         <v>50</v>
@@ -758,25 +758,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>40.4697</v>
+        <v>41.2313</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>40.4332</v>
+        <v>41.2396</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.3973</v>
+        <v>0.4023</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -802,25 +802,25 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>22.8954</v>
+        <v>23.1081</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1722</v>
+        <v>0.1998</v>
       </c>
       <c r="F8" t="n">
-        <v>21.9746</v>
+        <v>22.2472</v>
       </c>
       <c r="G8" t="n">
-        <v>0.2321</v>
+        <v>0.1896</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0.222</v>
+        <v>0.2244</v>
       </c>
       <c r="K8" t="n">
         <v>0.0004</v>
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6.4715</v>
+        <v>6.4238</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2277</v>
+        <v>0.1845</v>
       </c>
       <c r="F9" t="n">
-        <v>4.9435</v>
+        <v>5.033</v>
       </c>
       <c r="G9" t="n">
-        <v>0.4387</v>
+        <v>0.3169</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.6913</v>
       </c>
       <c r="I9" t="n">
         <v>0.0114</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1381</v>
+        <v>0.1399</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
       <c r="L9" t="n">
         <v>100</v>
@@ -890,28 +890,28 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>7.1169</v>
+        <v>7.0792</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2696</v>
+        <v>0.3051</v>
       </c>
       <c r="F10" t="n">
-        <v>5.9018</v>
+        <v>5.8869</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0993</v>
+        <v>0.1279</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.6915</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0111</v>
+        <v>0.0113</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1398</v>
+        <v>0.1415</v>
       </c>
       <c r="K10" t="n">
-        <v>0.0008</v>
+        <v>0.001</v>
       </c>
       <c r="L10" t="n">
         <v>100</v>
@@ -934,28 +934,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6.9172</v>
+        <v>6.8889</v>
       </c>
       <c r="E11" t="n">
-        <v>0.2377</v>
+        <v>0.1876</v>
       </c>
       <c r="F11" t="n">
-        <v>5.5052</v>
+        <v>5.5715</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4694</v>
+        <v>0.4307</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6854</v>
+        <v>0.6947</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0059</v>
+        <v>0.0057</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1375</v>
+        <v>0.1393</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0011</v>
+        <v>0.0009</v>
       </c>
       <c r="L11" t="n">
         <v>100</v>
@@ -978,25 +978,25 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>40.4697</v>
+        <v>41.2313</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>40.4332</v>
+        <v>41.2396</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.3973</v>
+        <v>0.4023</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -1022,28 +1022,28 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>22.8627</v>
+        <v>23.0549</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1289</v>
+        <v>0.1207</v>
       </c>
       <c r="F13" t="n">
-        <v>21.911</v>
+        <v>22.1465</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1012</v>
+        <v>0.0624</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0.2217</v>
+        <v>0.224</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
       <c r="L13" t="n">
         <v>200</v>
@@ -1066,25 +1066,25 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6.2002</v>
+        <v>6.0828</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0872</v>
+        <v>0.0704</v>
       </c>
       <c r="F14" t="n">
-        <v>4.649</v>
+        <v>4.6484</v>
       </c>
       <c r="G14" t="n">
-        <v>0.664</v>
+        <v>0.6768999999999999</v>
       </c>
       <c r="H14" t="n">
-        <v>0.6909999999999999</v>
+        <v>0.7003</v>
       </c>
       <c r="I14" t="n">
         <v>0.0032</v>
       </c>
       <c r="J14" t="n">
-        <v>0.1373</v>
+        <v>0.139</v>
       </c>
       <c r="K14" t="n">
         <v>0.0002</v>
@@ -1110,28 +1110,28 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6.55</v>
+        <v>6.4924</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2832</v>
+        <v>0.2428</v>
       </c>
       <c r="F15" t="n">
-        <v>5.0055</v>
+        <v>5.0732</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3596</v>
+        <v>0.2848</v>
       </c>
       <c r="H15" t="n">
-        <v>0.6912</v>
+        <v>0.7012</v>
       </c>
       <c r="I15" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.008399999999999999</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1368</v>
+        <v>0.1385</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="L15" t="n">
         <v>200</v>
@@ -1154,25 +1154,25 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6.4558</v>
+        <v>6.3697</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1926</v>
+        <v>0.1369</v>
       </c>
       <c r="F16" t="n">
-        <v>5.0288</v>
+        <v>5.0509</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4616</v>
+        <v>0.4507</v>
       </c>
       <c r="H16" t="n">
-        <v>0.6882</v>
+        <v>0.6977</v>
       </c>
       <c r="I16" t="n">
         <v>0.0012</v>
       </c>
       <c r="J16" t="n">
-        <v>0.1354</v>
+        <v>0.137</v>
       </c>
       <c r="K16" t="n">
         <v>0.0003</v>
@@ -1198,25 +1198,25 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>40.4697</v>
+        <v>41.2313</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>40.4332</v>
+        <v>41.2396</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3973</v>
+        <v>0.4023</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1242,28 +1242,28 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>22.8015</v>
+        <v>23.0045</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0371</v>
+        <v>0.0415</v>
       </c>
       <c r="F18" t="n">
-        <v>21.8362</v>
+        <v>22.1017</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0137</v>
+        <v>0.0381</v>
       </c>
       <c r="H18" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2215</v>
+        <v>0.2239</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L18" t="n">
         <v>500</v>
@@ -1286,25 +1286,25 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5.9416</v>
+        <v>5.8086</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1123</v>
+        <v>0.1144</v>
       </c>
       <c r="F19" t="n">
-        <v>4.0814</v>
+        <v>4.0781</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1714</v>
+        <v>0.179</v>
       </c>
       <c r="H19" t="n">
-        <v>0.6892</v>
+        <v>0.6985</v>
       </c>
       <c r="I19" t="n">
         <v>0.0011</v>
       </c>
       <c r="J19" t="n">
-        <v>0.1367</v>
+        <v>0.1384</v>
       </c>
       <c r="K19" t="n">
         <v>0.0003</v>
@@ -1330,28 +1330,28 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>6.0258</v>
+        <v>5.9714</v>
       </c>
       <c r="E20" t="n">
-        <v>0.2316</v>
+        <v>0.2565</v>
       </c>
       <c r="F20" t="n">
-        <v>4.6532</v>
+        <v>4.6766</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1447</v>
+        <v>0.1675</v>
       </c>
       <c r="H20" t="n">
-        <v>0.7033</v>
+        <v>0.7129</v>
       </c>
       <c r="I20" t="n">
-        <v>0.004</v>
+        <v>0.0038</v>
       </c>
       <c r="J20" t="n">
-        <v>0.1349</v>
+        <v>0.1365</v>
       </c>
       <c r="K20" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="L20" t="n">
         <v>500</v>
@@ -1374,28 +1374,28 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6.1998</v>
+        <v>6.1522</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2951</v>
+        <v>0.2369</v>
       </c>
       <c r="F21" t="n">
-        <v>4.5771</v>
+        <v>4.6492</v>
       </c>
       <c r="G21" t="n">
-        <v>0.2944</v>
+        <v>0.2846</v>
       </c>
       <c r="H21" t="n">
-        <v>0.6904</v>
+        <v>0.6998</v>
       </c>
       <c r="I21" t="n">
-        <v>0.0013</v>
+        <v>0.0012</v>
       </c>
       <c r="J21" t="n">
-        <v>0.1344</v>
+        <v>0.136</v>
       </c>
       <c r="K21" t="n">
-        <v>0.0002</v>
+        <v>0.0003</v>
       </c>
       <c r="L21" t="n">
         <v>500</v>
@@ -1418,25 +1418,25 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>40.4697</v>
+        <v>41.2313</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>40.4332</v>
+        <v>41.2396</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0.3973</v>
+        <v>0.4023</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -1462,25 +1462,25 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>22.8066</v>
+        <v>23.0086</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0211</v>
+        <v>0.0212</v>
       </c>
       <c r="F23" t="n">
-        <v>21.7912</v>
+        <v>22.0864</v>
       </c>
       <c r="G23" t="n">
-        <v>0.067</v>
+        <v>0.0561</v>
       </c>
       <c r="H23" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0.2216</v>
+        <v>0.2239</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -1506,25 +1506,25 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5.8546</v>
+        <v>5.7047</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0629</v>
+        <v>0.0672</v>
       </c>
       <c r="F24" t="n">
-        <v>3.8808</v>
+        <v>3.8894</v>
       </c>
       <c r="G24" t="n">
-        <v>0.128</v>
+        <v>0.1076</v>
       </c>
       <c r="H24" t="n">
-        <v>0.6892</v>
+        <v>0.6985</v>
       </c>
       <c r="I24" t="n">
         <v>0.0011</v>
       </c>
       <c r="J24" t="n">
-        <v>0.1366</v>
+        <v>0.1383</v>
       </c>
       <c r="K24" t="n">
         <v>0.0001</v>
@@ -1550,25 +1550,25 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>5.9902</v>
+        <v>5.8969</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0825</v>
+        <v>0.0609</v>
       </c>
       <c r="F25" t="n">
-        <v>4.5003</v>
+        <v>4.5311</v>
       </c>
       <c r="G25" t="n">
-        <v>0.1461</v>
+        <v>0.1757</v>
       </c>
       <c r="H25" t="n">
-        <v>0.7084</v>
+        <v>0.7183</v>
       </c>
       <c r="I25" t="n">
-        <v>0.0032</v>
+        <v>0.0033</v>
       </c>
       <c r="J25" t="n">
-        <v>0.1343</v>
+        <v>0.1359</v>
       </c>
       <c r="K25" t="n">
         <v>0.0004</v>
@@ -1594,25 +1594,25 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5.915</v>
+        <v>5.864</v>
       </c>
       <c r="E26" t="n">
-        <v>0.136</v>
+        <v>0.1279</v>
       </c>
       <c r="F26" t="n">
-        <v>4.0867</v>
+        <v>4.1525</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1026</v>
+        <v>0.1226</v>
       </c>
       <c r="H26" t="n">
-        <v>0.6913</v>
+        <v>0.7007</v>
       </c>
       <c r="I26" t="n">
         <v>0.0005999999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1341</v>
+        <v>0.1358</v>
       </c>
       <c r="K26" t="n">
         <v>0.0003</v>
@@ -1638,25 +1638,25 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>40.4697</v>
+        <v>41.2313</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>40.4332</v>
+        <v>41.2396</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0.3973</v>
+        <v>0.4023</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -1682,25 +1682,25 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>22.8065</v>
+        <v>23.0101</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0081</v>
+        <v>0.0083</v>
       </c>
       <c r="F28" t="n">
-        <v>21.8405</v>
+        <v>22.1304</v>
       </c>
       <c r="G28" t="n">
-        <v>0.0363</v>
+        <v>0.0385</v>
       </c>
       <c r="H28" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0.2216</v>
+        <v>0.2239</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -1726,25 +1726,25 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5.8283</v>
+        <v>5.6909</v>
       </c>
       <c r="E29" t="n">
-        <v>0.0066</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="F29" t="n">
-        <v>3.8899</v>
+        <v>3.8419</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1</v>
+        <v>0.08119999999999999</v>
       </c>
       <c r="H29" t="n">
-        <v>0.6887</v>
+        <v>0.698</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0.1366</v>
+        <v>0.1383</v>
       </c>
       <c r="K29" t="n">
         <v>0.0001</v>
@@ -1770,25 +1770,25 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>6.0989</v>
+        <v>5.9911</v>
       </c>
       <c r="E30" t="n">
-        <v>0.1234</v>
+        <v>0.1181</v>
       </c>
       <c r="F30" t="n">
-        <v>4.6566</v>
+        <v>4.6814</v>
       </c>
       <c r="G30" t="n">
-        <v>0.0964</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="H30" t="n">
-        <v>0.7099</v>
+        <v>0.7201</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0008</v>
+        <v>0.0009</v>
       </c>
       <c r="J30" t="n">
-        <v>0.1341</v>
+        <v>0.1356</v>
       </c>
       <c r="K30" t="n">
         <v>0.0001</v>
@@ -1814,25 +1814,25 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6.162</v>
+        <v>6.091</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0781</v>
+        <v>0.0891</v>
       </c>
       <c r="F31" t="n">
-        <v>4.2652</v>
+        <v>4.3094</v>
       </c>
       <c r="G31" t="n">
-        <v>0.068</v>
+        <v>0.08450000000000001</v>
       </c>
       <c r="H31" t="n">
-        <v>0.6912</v>
+        <v>0.7008</v>
       </c>
       <c r="I31" t="n">
         <v>0.0004</v>
       </c>
       <c r="J31" t="n">
-        <v>0.1343</v>
+        <v>0.1359</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1858,25 +1858,25 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>40.4697</v>
+        <v>41.2313</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>40.4332</v>
+        <v>41.2396</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>0.3973</v>
+        <v>0.4023</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1902,25 +1902,25 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>22.8112</v>
+        <v>23.0146</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>21.9188</v>
+        <v>22.1877</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0.6649</v>
+        <v>0.6742</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0.2216</v>
+        <v>0.2239</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -1946,25 +1946,25 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5.8298</v>
+        <v>5.6927</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>3.9731</v>
+        <v>3.9037</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0.6887</v>
+        <v>0.698</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0.1366</v>
+        <v>0.1383</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -1990,25 +1990,25 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>6.0967</v>
+        <v>5.8519</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>4.8055</v>
+        <v>4.7714</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0.71</v>
+        <v>0.7202</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>0.134</v>
+        <v>0.1356</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -2034,25 +2034,25 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>6.3035</v>
+        <v>6.167</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>4.2432</v>
+        <v>4.2981</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0.6911</v>
+        <v>0.7006</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0.1343</v>
+        <v>0.1359</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -7102,25 +7102,25 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>11.2643</v>
+        <v>21.9267</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>10.8682</v>
+        <v>22.1575</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0.1669</v>
+        <v>0.2368</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
@@ -7148,28 +7148,28 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>10.0683</v>
+        <v>12.9168</v>
       </c>
       <c r="F3" t="n">
-        <v>0.205</v>
+        <v>0.3403</v>
       </c>
       <c r="G3" t="n">
-        <v>10.189</v>
+        <v>13.1928</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3782</v>
+        <v>0.5228</v>
       </c>
       <c r="I3" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0.1596</v>
+        <v>0.1926</v>
       </c>
       <c r="L3" t="n">
-        <v>0.0007</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="4">
@@ -7194,28 +7194,28 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>7.8267</v>
+        <v>7.1742</v>
       </c>
       <c r="F4" t="n">
-        <v>1.5829</v>
+        <v>2.301</v>
       </c>
       <c r="G4" t="n">
-        <v>6.3546</v>
+        <v>7.9871</v>
       </c>
       <c r="H4" t="n">
-        <v>1.814</v>
+        <v>2.0939</v>
       </c>
       <c r="I4" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1524</v>
+        <v>0.1772</v>
       </c>
       <c r="L4" t="n">
-        <v>0.0056</v>
+        <v>0.0043</v>
       </c>
     </row>
     <row r="5">
@@ -7240,28 +7240,28 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>9.3529</v>
+        <v>8.854900000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>2.384</v>
+        <v>1.6844</v>
       </c>
       <c r="G5" t="n">
-        <v>8.496</v>
+        <v>8.565099999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>3.0004</v>
+        <v>2.4105</v>
       </c>
       <c r="I5" t="n">
-        <v>0.651</v>
+        <v>0.7874</v>
       </c>
       <c r="J5" t="n">
-        <v>0.0404</v>
+        <v>0.0108</v>
       </c>
       <c r="K5" t="n">
-        <v>0.161</v>
+        <v>0.1863</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0108</v>
+        <v>0.0059</v>
       </c>
     </row>
     <row r="6">
@@ -7286,28 +7286,28 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>8.2683</v>
+        <v>7.7269</v>
       </c>
       <c r="F6" t="n">
-        <v>1.8729</v>
+        <v>2.2514</v>
       </c>
       <c r="G6" t="n">
-        <v>7.4833</v>
+        <v>7.9153</v>
       </c>
       <c r="H6" t="n">
-        <v>2.3679</v>
+        <v>2.9589</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6761</v>
+        <v>0.8066</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0042</v>
+        <v>0.0031</v>
       </c>
       <c r="K6" t="n">
-        <v>0.1541</v>
+        <v>0.1784</v>
       </c>
       <c r="L6" t="n">
-        <v>0.0072</v>
+        <v>0.0071</v>
       </c>
     </row>
     <row r="7">
@@ -7332,25 +7332,25 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>11.2643</v>
+        <v>21.9267</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>10.8682</v>
+        <v>22.1575</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0.1669</v>
+        <v>0.2368</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
@@ -7378,28 +7378,28 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>9.999599999999999</v>
+        <v>12.9775</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1201</v>
+        <v>0.5358000000000001</v>
       </c>
       <c r="G8" t="n">
-        <v>9.2706</v>
+        <v>13.0873</v>
       </c>
       <c r="H8" t="n">
-        <v>0.579</v>
+        <v>0.2254</v>
       </c>
       <c r="I8" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.1594</v>
+        <v>0.1929</v>
       </c>
       <c r="L8" t="n">
-        <v>0.0003</v>
+        <v>0.0013</v>
       </c>
     </row>
     <row r="9">
@@ -7424,28 +7424,28 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>7.4011</v>
+        <v>6.733</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6599</v>
+        <v>2.5517</v>
       </c>
       <c r="G9" t="n">
-        <v>5.8907</v>
+        <v>7.1432</v>
       </c>
       <c r="H9" t="n">
-        <v>1.6272</v>
+        <v>1.9641</v>
       </c>
       <c r="I9" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1512</v>
+        <v>0.1767</v>
       </c>
       <c r="L9" t="n">
-        <v>0.0018</v>
+        <v>0.0048</v>
       </c>
     </row>
     <row r="10">
@@ -7470,28 +7470,28 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>7.9767</v>
+        <v>7.45</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9188</v>
+        <v>0.5891999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>7.6662</v>
+        <v>7.4586</v>
       </c>
       <c r="H10" t="n">
-        <v>1.1078</v>
+        <v>0.5685</v>
       </c>
       <c r="I10" t="n">
-        <v>0.6621</v>
+        <v>0.7948</v>
       </c>
       <c r="J10" t="n">
-        <v>0.0275</v>
+        <v>0.0231</v>
       </c>
       <c r="K10" t="n">
-        <v>0.1567</v>
+        <v>0.1803</v>
       </c>
       <c r="L10" t="n">
-        <v>0.005</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="11">
@@ -7516,28 +7516,28 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>8.079599999999999</v>
+        <v>7.684</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7803</v>
+        <v>1.4813</v>
       </c>
       <c r="G11" t="n">
-        <v>6.7268</v>
+        <v>7.6554</v>
       </c>
       <c r="H11" t="n">
-        <v>0.9375</v>
+        <v>1.3175</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6768</v>
+        <v>0.8073</v>
       </c>
       <c r="J11" t="n">
-        <v>0.003</v>
+        <v>0.0022</v>
       </c>
       <c r="K11" t="n">
-        <v>0.1518</v>
+        <v>0.1768</v>
       </c>
       <c r="L11" t="n">
-        <v>0.0015</v>
+        <v>0.0039</v>
       </c>
     </row>
     <row r="12">
@@ -7562,25 +7562,25 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>11.2643</v>
+        <v>21.9267</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>10.8682</v>
+        <v>22.1575</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>0.1669</v>
+        <v>0.2368</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
@@ -7608,28 +7608,28 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>10.0277</v>
+        <v>12.7184</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1918</v>
+        <v>0.0603</v>
       </c>
       <c r="G13" t="n">
-        <v>9.761699999999999</v>
+        <v>13.0591</v>
       </c>
       <c r="H13" t="n">
-        <v>0.4176</v>
+        <v>0.2961</v>
       </c>
       <c r="I13" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0.1595</v>
+        <v>0.1924</v>
       </c>
       <c r="L13" t="n">
-        <v>0.0005</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="14">
@@ -7654,28 +7654,28 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>7.27</v>
+        <v>5.6268</v>
       </c>
       <c r="F14" t="n">
-        <v>0.353</v>
+        <v>0.4757</v>
       </c>
       <c r="G14" t="n">
-        <v>6.1574</v>
+        <v>6.1491</v>
       </c>
       <c r="H14" t="n">
-        <v>0.437</v>
+        <v>0.8421999999999999</v>
       </c>
       <c r="I14" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0.1508</v>
+        <v>0.1742</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0016</v>
+        <v>0.0009</v>
       </c>
     </row>
     <row r="15">
@@ -7700,28 +7700,28 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>7.7553</v>
+        <v>6.9495</v>
       </c>
       <c r="F15" t="n">
-        <v>1.0697</v>
+        <v>0.8183</v>
       </c>
       <c r="G15" t="n">
-        <v>5.6131</v>
+        <v>6.5617</v>
       </c>
       <c r="H15" t="n">
-        <v>1.1131</v>
+        <v>1.2885</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6618000000000001</v>
+        <v>0.8021</v>
       </c>
       <c r="J15" t="n">
-        <v>0.017</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="K15" t="n">
-        <v>0.1541</v>
+        <v>0.1771</v>
       </c>
       <c r="L15" t="n">
-        <v>0.003</v>
+        <v>0.0029</v>
       </c>
     </row>
     <row r="16">
@@ -7746,28 +7746,28 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>8.0319</v>
+        <v>6.8269</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7809</v>
+        <v>0.7485000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>6.5823</v>
+        <v>6.8914</v>
       </c>
       <c r="H16" t="n">
-        <v>1.4246</v>
+        <v>0.9704</v>
       </c>
       <c r="I16" t="n">
-        <v>0.6747</v>
+        <v>0.8086</v>
       </c>
       <c r="J16" t="n">
-        <v>0.0035</v>
+        <v>0.001</v>
       </c>
       <c r="K16" t="n">
-        <v>0.1515</v>
+        <v>0.174</v>
       </c>
       <c r="L16" t="n">
-        <v>0.0021</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="17">
@@ -7792,25 +7792,25 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>11.2643</v>
+        <v>21.9267</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>10.8682</v>
+        <v>22.1575</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1669</v>
+        <v>0.2368</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
@@ -7838,28 +7838,28 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>9.882999999999999</v>
+        <v>12.7246</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0389</v>
+        <v>0.0704</v>
       </c>
       <c r="G18" t="n">
-        <v>9.2455</v>
+        <v>12.9619</v>
       </c>
       <c r="H18" t="n">
-        <v>0.2908</v>
+        <v>0.2644</v>
       </c>
       <c r="I18" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0.1591</v>
+        <v>0.1924</v>
       </c>
       <c r="L18" t="n">
-        <v>0.0001</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -7884,28 +7884,28 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>7.0167</v>
+        <v>5.1543</v>
       </c>
       <c r="F19" t="n">
-        <v>0.1426</v>
+        <v>0.1341</v>
       </c>
       <c r="G19" t="n">
-        <v>5.8121</v>
+        <v>5.7656</v>
       </c>
       <c r="H19" t="n">
-        <v>0.6585</v>
+        <v>0.7208</v>
       </c>
       <c r="I19" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0.1498</v>
+        <v>0.1733</v>
       </c>
       <c r="L19" t="n">
-        <v>0.0007</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="20">
@@ -7930,28 +7930,28 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>7.4598</v>
+        <v>6.6988</v>
       </c>
       <c r="F20" t="n">
-        <v>0.6413</v>
+        <v>1.1721</v>
       </c>
       <c r="G20" t="n">
-        <v>6.0852</v>
+        <v>6.4136</v>
       </c>
       <c r="H20" t="n">
-        <v>1.0143</v>
+        <v>1.143</v>
       </c>
       <c r="I20" t="n">
-        <v>0.6758999999999999</v>
+        <v>0.8109</v>
       </c>
       <c r="J20" t="n">
-        <v>0.0152</v>
+        <v>0.0024</v>
       </c>
       <c r="K20" t="n">
-        <v>0.1505</v>
+        <v>0.173</v>
       </c>
       <c r="L20" t="n">
-        <v>0.0016</v>
+        <v>0.0011</v>
       </c>
     </row>
     <row r="21">
@@ -7976,28 +7976,28 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>7.1315</v>
+        <v>6.4659</v>
       </c>
       <c r="F21" t="n">
-        <v>0.8247</v>
+        <v>0.7772</v>
       </c>
       <c r="G21" t="n">
-        <v>5.306</v>
+        <v>6.315</v>
       </c>
       <c r="H21" t="n">
-        <v>1.2738</v>
+        <v>0.5551</v>
       </c>
       <c r="I21" t="n">
-        <v>0.6776</v>
+        <v>0.8095</v>
       </c>
       <c r="J21" t="n">
-        <v>0.0028</v>
+        <v>0.0007</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1497</v>
+        <v>0.1726</v>
       </c>
       <c r="L21" t="n">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
     </row>
     <row r="22">
@@ -8022,25 +8022,25 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>11.2643</v>
+        <v>21.9267</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
       </c>
       <c r="G22" t="n">
-        <v>10.8682</v>
+        <v>22.1575</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>0.1669</v>
+        <v>0.2368</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
@@ -8068,28 +8068,28 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>9.854200000000001</v>
+        <v>12.6816</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0165</v>
+        <v>0.0067</v>
       </c>
       <c r="G23" t="n">
-        <v>9.17</v>
+        <v>13.3037</v>
       </c>
       <c r="H23" t="n">
-        <v>0.284</v>
+        <v>0.1778</v>
       </c>
       <c r="I23" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>0.159</v>
+        <v>0.1924</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="24">
@@ -8114,28 +8114,28 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>6.9124</v>
+        <v>4.8141</v>
       </c>
       <c r="F24" t="n">
-        <v>0.031</v>
+        <v>0.07240000000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>5.702</v>
+        <v>5.8235</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1922</v>
+        <v>0.3412</v>
       </c>
       <c r="I24" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0.1494</v>
+        <v>0.1731</v>
       </c>
       <c r="L24" t="n">
-        <v>0.0003</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="25">
@@ -8160,28 +8160,28 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>7.4945</v>
+        <v>6.1881</v>
       </c>
       <c r="F25" t="n">
-        <v>0.5778</v>
+        <v>0.6309</v>
       </c>
       <c r="G25" t="n">
-        <v>4.8793</v>
+        <v>5.3099</v>
       </c>
       <c r="H25" t="n">
-        <v>0.3257</v>
+        <v>0.272</v>
       </c>
       <c r="I25" t="n">
-        <v>0.6727</v>
+        <v>0.8121</v>
       </c>
       <c r="J25" t="n">
-        <v>0.0077</v>
+        <v>0.0015</v>
       </c>
       <c r="K25" t="n">
-        <v>0.1497</v>
+        <v>0.1721</v>
       </c>
       <c r="L25" t="n">
-        <v>0.0011</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="26">
@@ -8206,28 +8206,28 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>7.007</v>
+        <v>6.2935</v>
       </c>
       <c r="F26" t="n">
-        <v>0.3136</v>
+        <v>0.4882</v>
       </c>
       <c r="G26" t="n">
-        <v>4.6147</v>
+        <v>5.5347</v>
       </c>
       <c r="H26" t="n">
-        <v>0.2109</v>
+        <v>0.5</v>
       </c>
       <c r="I26" t="n">
-        <v>0.6774</v>
+        <v>0.8096</v>
       </c>
       <c r="J26" t="n">
-        <v>0.0015</v>
+        <v>0.0004</v>
       </c>
       <c r="K26" t="n">
-        <v>0.1493</v>
+        <v>0.1723</v>
       </c>
       <c r="L26" t="n">
-        <v>0.0004</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="27">
@@ -8252,25 +8252,25 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>11.2643</v>
+        <v>21.9267</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
       </c>
       <c r="G27" t="n">
-        <v>10.8682</v>
+        <v>22.1575</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>0.1669</v>
+        <v>0.2368</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
@@ -8298,28 +8298,28 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>9.833299999999999</v>
+        <v>12.6828</v>
       </c>
       <c r="F28" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.005</v>
       </c>
       <c r="G28" t="n">
-        <v>9.149699999999999</v>
+        <v>13.2072</v>
       </c>
       <c r="H28" t="n">
-        <v>0.1685</v>
+        <v>0.1971</v>
       </c>
       <c r="I28" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>0.159</v>
+        <v>0.1924</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="29">
@@ -8344,25 +8344,25 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>6.9077</v>
+        <v>4.9843</v>
       </c>
       <c r="F29" t="n">
-        <v>0.0055</v>
+        <v>0.0466</v>
       </c>
       <c r="G29" t="n">
-        <v>5.6018</v>
+        <v>4.9294</v>
       </c>
       <c r="H29" t="n">
-        <v>0.3395</v>
+        <v>0.3612</v>
       </c>
       <c r="I29" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
       </c>
       <c r="K29" t="n">
-        <v>0.1493</v>
+        <v>0.1732</v>
       </c>
       <c r="L29" t="n">
         <v>0.0001</v>
@@ -8390,28 +8390,28 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>8.102600000000001</v>
+        <v>6.5934</v>
       </c>
       <c r="F30" t="n">
-        <v>0.5305</v>
+        <v>0.4931</v>
       </c>
       <c r="G30" t="n">
-        <v>5.3203</v>
+        <v>5.6681</v>
       </c>
       <c r="H30" t="n">
-        <v>0.1652</v>
+        <v>0.378</v>
       </c>
       <c r="I30" t="n">
-        <v>0.6697</v>
+        <v>0.8128</v>
       </c>
       <c r="J30" t="n">
-        <v>0.0019</v>
+        <v>0.0003</v>
       </c>
       <c r="K30" t="n">
-        <v>0.1501</v>
+        <v>0.1719</v>
       </c>
       <c r="L30" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="31">
@@ -8436,25 +8436,25 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>7.0241</v>
+        <v>6.0296</v>
       </c>
       <c r="F31" t="n">
-        <v>0.4362</v>
+        <v>0.1647</v>
       </c>
       <c r="G31" t="n">
-        <v>4.9519</v>
+        <v>5.5707</v>
       </c>
       <c r="H31" t="n">
-        <v>0.4223</v>
+        <v>0.1799</v>
       </c>
       <c r="I31" t="n">
-        <v>0.6764</v>
+        <v>0.8099</v>
       </c>
       <c r="J31" t="n">
-        <v>0.0005</v>
+        <v>0.0003</v>
       </c>
       <c r="K31" t="n">
-        <v>0.1493</v>
+        <v>0.1723</v>
       </c>
       <c r="L31" t="n">
         <v>0.0001</v>
@@ -8482,25 +8482,25 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>11.2643</v>
+        <v>21.9267</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
       </c>
       <c r="G32" t="n">
-        <v>10.8682</v>
+        <v>22.1575</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J32" t="n">
         <v>0</v>
       </c>
       <c r="K32" t="n">
-        <v>0.1669</v>
+        <v>0.2368</v>
       </c>
       <c r="L32" t="n">
         <v>0</v>
@@ -8528,25 +8528,25 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>9.833600000000001</v>
+        <v>12.6817</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
       </c>
       <c r="G33" t="n">
-        <v>9.3338</v>
+        <v>13.0988</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>0.159</v>
+        <v>0.1924</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
@@ -8574,25 +8574,25 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>6.9058</v>
+        <v>4.9865</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>5.7702</v>
+        <v>4.7986</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>0.677</v>
+        <v>0.8067</v>
       </c>
       <c r="J34" t="n">
         <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>0.1492</v>
+        <v>0.1732</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
@@ -8620,25 +8620,25 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>9.581899999999999</v>
+        <v>6.1545</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>5.6483</v>
+        <v>5.1709</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
       </c>
       <c r="I35" t="n">
-        <v>0.6699000000000001</v>
+        <v>0.8128</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0.1499</v>
+        <v>0.1719</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
@@ -8666,25 +8666,25 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>7.672</v>
+        <v>5.7612</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
       </c>
       <c r="G36" t="n">
-        <v>4.9048</v>
+        <v>5.6727</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
       </c>
       <c r="I36" t="n">
-        <v>0.6766</v>
+        <v>0.8099</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>0.1491</v>
+        <v>0.1723</v>
       </c>
       <c r="L36" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat(tables): transition to Core 5 benchmarks, update transfer targets, and targeted sample efficiency
</commit_message>
<xml_diff>
--- a/sheets/sample_efficiency_results.xlsx
+++ b/sheets/sample_efficiency_results.xlsx
@@ -538,25 +538,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>41.2313</v>
+        <v>19.6401</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>41.2396</v>
+        <v>19.8536</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4023</v>
+        <v>0.2348</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -582,28 +582,28 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>23.1856</v>
+        <v>12.277</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1537</v>
+        <v>0.4745</v>
       </c>
       <c r="F3" t="n">
-        <v>22.4249</v>
+        <v>11.755</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1778</v>
+        <v>0.4722</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0.2245</v>
+        <v>0.1933</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0005</v>
+        <v>0.0014</v>
       </c>
       <c r="L3" t="n">
         <v>50</v>
@@ -626,28 +626,28 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6.9268</v>
+        <v>7.7173</v>
       </c>
       <c r="E4" t="n">
-        <v>0.495</v>
+        <v>0.7909</v>
       </c>
       <c r="F4" t="n">
-        <v>5.6404</v>
+        <v>7.119</v>
       </c>
       <c r="G4" t="n">
-        <v>0.7389</v>
+        <v>0.8974</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6937</v>
+        <v>0.765</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0116</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>0.1413</v>
+        <v>0.1809</v>
       </c>
       <c r="K4" t="n">
-        <v>0.0014</v>
+        <v>0.002</v>
       </c>
       <c r="L4" t="n">
         <v>50</v>
@@ -670,28 +670,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>7.5806</v>
+        <v>8.6408</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5078</v>
+        <v>1.4286</v>
       </c>
       <c r="F5" t="n">
-        <v>6.7904</v>
+        <v>8.241</v>
       </c>
       <c r="G5" t="n">
-        <v>0.5952</v>
+        <v>1.4243</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6737</v>
+        <v>0.7422</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0138</v>
+        <v>0.0165</v>
       </c>
       <c r="J5" t="n">
-        <v>0.1456</v>
+        <v>0.1897</v>
       </c>
       <c r="K5" t="n">
-        <v>0.001</v>
+        <v>0.0047</v>
       </c>
       <c r="L5" t="n">
         <v>50</v>
@@ -714,28 +714,28 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>7.9243</v>
+        <v>9.1043</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4453</v>
+        <v>0.6314</v>
       </c>
       <c r="F6" t="n">
-        <v>6.9042</v>
+        <v>8.8116</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8883</v>
+        <v>0.9024</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6874</v>
+        <v>0.7678</v>
       </c>
       <c r="I6" t="n">
-        <v>0.011</v>
+        <v>0.015</v>
       </c>
       <c r="J6" t="n">
-        <v>0.1445</v>
+        <v>0.1825</v>
       </c>
       <c r="K6" t="n">
-        <v>0.0027</v>
+        <v>0.0054</v>
       </c>
       <c r="L6" t="n">
         <v>50</v>
@@ -758,25 +758,25 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>41.2313</v>
+        <v>19.6401</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>41.2396</v>
+        <v>19.8536</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0.4023</v>
+        <v>0.2348</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -802,28 +802,28 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>23.1081</v>
+        <v>12.1585</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1998</v>
+        <v>0.5738</v>
       </c>
       <c r="F8" t="n">
-        <v>22.2472</v>
+        <v>11.5352</v>
       </c>
       <c r="G8" t="n">
-        <v>0.1896</v>
+        <v>0.3868</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>0.2244</v>
+        <v>0.193</v>
       </c>
       <c r="K8" t="n">
-        <v>0.0004</v>
+        <v>0.0011</v>
       </c>
       <c r="L8" t="n">
         <v>100</v>
@@ -846,28 +846,28 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6.4238</v>
+        <v>7.548</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1845</v>
+        <v>0.7379</v>
       </c>
       <c r="F9" t="n">
-        <v>5.033</v>
+        <v>6.9658</v>
       </c>
       <c r="G9" t="n">
-        <v>0.3169</v>
+        <v>0.71</v>
       </c>
       <c r="H9" t="n">
-        <v>0.6913</v>
+        <v>0.765</v>
       </c>
       <c r="I9" t="n">
-        <v>0.0114</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1399</v>
+        <v>0.1805</v>
       </c>
       <c r="K9" t="n">
-        <v>0.0008</v>
+        <v>0.0024</v>
       </c>
       <c r="L9" t="n">
         <v>100</v>
@@ -890,28 +890,28 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>7.0792</v>
+        <v>7.8587</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3051</v>
+        <v>0.7325</v>
       </c>
       <c r="F10" t="n">
-        <v>5.8869</v>
+        <v>7.4302</v>
       </c>
       <c r="G10" t="n">
-        <v>0.1279</v>
+        <v>0.8149</v>
       </c>
       <c r="H10" t="n">
-        <v>0.6915</v>
+        <v>0.7606000000000001</v>
       </c>
       <c r="I10" t="n">
-        <v>0.0113</v>
+        <v>0.015</v>
       </c>
       <c r="J10" t="n">
-        <v>0.1415</v>
+        <v>0.1827</v>
       </c>
       <c r="K10" t="n">
-        <v>0.001</v>
+        <v>0.0035</v>
       </c>
       <c r="L10" t="n">
         <v>100</v>
@@ -934,28 +934,28 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6.8889</v>
+        <v>8.1808</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1876</v>
+        <v>0.6209</v>
       </c>
       <c r="F11" t="n">
-        <v>5.5715</v>
+        <v>7.6285</v>
       </c>
       <c r="G11" t="n">
-        <v>0.4307</v>
+        <v>0.3315</v>
       </c>
       <c r="H11" t="n">
-        <v>0.6947</v>
+        <v>0.7708</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0057</v>
+        <v>0.008699999999999999</v>
       </c>
       <c r="J11" t="n">
-        <v>0.1393</v>
+        <v>0.1795</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0009</v>
+        <v>0.001</v>
       </c>
       <c r="L11" t="n">
         <v>100</v>
@@ -978,25 +978,25 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>41.2313</v>
+        <v>19.6401</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>41.2396</v>
+        <v>19.8536</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0.4023</v>
+        <v>0.2348</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -1022,28 +1022,28 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>23.0549</v>
+        <v>12.0341</v>
       </c>
       <c r="E13" t="n">
-        <v>0.1207</v>
+        <v>0.3496</v>
       </c>
       <c r="F13" t="n">
-        <v>22.1465</v>
+        <v>11.4916</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0624</v>
+        <v>0.2582</v>
       </c>
       <c r="H13" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0.224</v>
+        <v>0.1921</v>
       </c>
       <c r="K13" t="n">
-        <v>0.0002</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="L13" t="n">
         <v>200</v>
@@ -1066,28 +1066,28 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6.0828</v>
+        <v>7.1756</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0704</v>
+        <v>0.2303</v>
       </c>
       <c r="F14" t="n">
-        <v>4.6484</v>
+        <v>6.5152</v>
       </c>
       <c r="G14" t="n">
-        <v>0.6768999999999999</v>
+        <v>0.2695</v>
       </c>
       <c r="H14" t="n">
-        <v>0.7003</v>
+        <v>0.765</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0032</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>0.139</v>
+        <v>0.1796</v>
       </c>
       <c r="K14" t="n">
-        <v>0.0002</v>
+        <v>0.0009</v>
       </c>
       <c r="L14" t="n">
         <v>200</v>
@@ -1110,28 +1110,28 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>6.4924</v>
+        <v>7.5835</v>
       </c>
       <c r="E15" t="n">
-        <v>0.2428</v>
+        <v>0.4228</v>
       </c>
       <c r="F15" t="n">
-        <v>5.0732</v>
+        <v>6.7196</v>
       </c>
       <c r="G15" t="n">
-        <v>0.2848</v>
+        <v>0.2975</v>
       </c>
       <c r="H15" t="n">
-        <v>0.7012</v>
+        <v>0.7708</v>
       </c>
       <c r="I15" t="n">
-        <v>0.008399999999999999</v>
+        <v>0.0072</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1385</v>
+        <v>0.18</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0008</v>
+        <v>0.0018</v>
       </c>
       <c r="L15" t="n">
         <v>200</v>
@@ -1154,28 +1154,28 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>6.3697</v>
+        <v>7.8043</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1369</v>
+        <v>0.3977</v>
       </c>
       <c r="F16" t="n">
-        <v>5.0509</v>
+        <v>6.9439</v>
       </c>
       <c r="G16" t="n">
-        <v>0.4507</v>
+        <v>0.3536</v>
       </c>
       <c r="H16" t="n">
-        <v>0.6977</v>
+        <v>0.7756999999999999</v>
       </c>
       <c r="I16" t="n">
+        <v>0.0038</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.1775</v>
+      </c>
+      <c r="K16" t="n">
         <v>0.0012</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0.137</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0.0003</v>
       </c>
       <c r="L16" t="n">
         <v>200</v>
@@ -1198,25 +1198,25 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>41.2313</v>
+        <v>19.6401</v>
       </c>
       <c r="E17" t="n">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>41.2396</v>
+        <v>19.8536</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
       </c>
       <c r="H17" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0.4023</v>
+        <v>0.2348</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -1242,25 +1242,25 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>23.0045</v>
+        <v>11.9028</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0415</v>
+        <v>0.1141</v>
       </c>
       <c r="F18" t="n">
-        <v>22.1017</v>
+        <v>11.3036</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0381</v>
+        <v>0.1223</v>
       </c>
       <c r="H18" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2239</v>
+        <v>0.1918</v>
       </c>
       <c r="K18" t="n">
         <v>0.0001</v>
@@ -1286,28 +1286,28 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>5.8086</v>
+        <v>6.8286</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1144</v>
+        <v>0.1795</v>
       </c>
       <c r="F19" t="n">
-        <v>4.0781</v>
+        <v>6.2603</v>
       </c>
       <c r="G19" t="n">
-        <v>0.179</v>
+        <v>0.2744</v>
       </c>
       <c r="H19" t="n">
-        <v>0.6985</v>
+        <v>0.765</v>
       </c>
       <c r="I19" t="n">
-        <v>0.0011</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0.1384</v>
+        <v>0.1788</v>
       </c>
       <c r="K19" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
       <c r="L19" t="n">
         <v>500</v>
@@ -1330,28 +1330,28 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>5.9714</v>
+        <v>7.2096</v>
       </c>
       <c r="E20" t="n">
-        <v>0.2565</v>
+        <v>0.3172</v>
       </c>
       <c r="F20" t="n">
-        <v>4.6766</v>
+        <v>6.9628</v>
       </c>
       <c r="G20" t="n">
-        <v>0.1675</v>
+        <v>0.4065</v>
       </c>
       <c r="H20" t="n">
-        <v>0.7129</v>
+        <v>0.777</v>
       </c>
       <c r="I20" t="n">
-        <v>0.0038</v>
+        <v>0.0026</v>
       </c>
       <c r="J20" t="n">
-        <v>0.1365</v>
+        <v>0.1776</v>
       </c>
       <c r="K20" t="n">
-        <v>0.0003</v>
+        <v>0.0013</v>
       </c>
       <c r="L20" t="n">
         <v>500</v>
@@ -1374,25 +1374,25 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>6.1522</v>
+        <v>7.7672</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2369</v>
+        <v>0.5616</v>
       </c>
       <c r="F21" t="n">
-        <v>4.6492</v>
+        <v>6.5892</v>
       </c>
       <c r="G21" t="n">
-        <v>0.2846</v>
+        <v>0.2562</v>
       </c>
       <c r="H21" t="n">
-        <v>0.6998</v>
+        <v>0.7766999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>0.0012</v>
+        <v>0.0013</v>
       </c>
       <c r="J21" t="n">
-        <v>0.136</v>
+        <v>0.1764</v>
       </c>
       <c r="K21" t="n">
         <v>0.0003</v>
@@ -1418,31 +1418,31 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>41.2313</v>
+        <v>19.6401</v>
       </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>41.2396</v>
+        <v>19.8536</v>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I22" t="n">
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0.4023</v>
+        <v>0.2348</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>968.9</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="23">
@@ -1462,31 +1462,31 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>23.0086</v>
+        <v>11.916</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0212</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="F23" t="n">
-        <v>22.0864</v>
+        <v>11.2872</v>
       </c>
       <c r="G23" t="n">
-        <v>0.0561</v>
+        <v>0.1077</v>
       </c>
       <c r="H23" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I23" t="n">
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0.2239</v>
+        <v>0.1919</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L23" t="n">
-        <v>968.9</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="24">
@@ -1506,31 +1506,31 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>5.7047</v>
+        <v>6.6768</v>
       </c>
       <c r="E24" t="n">
-        <v>0.0672</v>
+        <v>0.095</v>
       </c>
       <c r="F24" t="n">
-        <v>3.8894</v>
+        <v>6.246</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1076</v>
+        <v>0.1601</v>
       </c>
       <c r="H24" t="n">
-        <v>0.6985</v>
+        <v>0.765</v>
       </c>
       <c r="I24" t="n">
-        <v>0.0011</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0.1383</v>
+        <v>0.1787</v>
       </c>
       <c r="K24" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="L24" t="n">
-        <v>968.9</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="25">
@@ -1550,31 +1550,31 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>5.8969</v>
+        <v>7.4745</v>
       </c>
       <c r="E25" t="n">
-        <v>0.0609</v>
+        <v>0.2347</v>
       </c>
       <c r="F25" t="n">
-        <v>4.5311</v>
+        <v>6.4641</v>
       </c>
       <c r="G25" t="n">
-        <v>0.1757</v>
+        <v>0.1975</v>
       </c>
       <c r="H25" t="n">
-        <v>0.7183</v>
+        <v>0.7774</v>
       </c>
       <c r="I25" t="n">
-        <v>0.0033</v>
+        <v>0.002</v>
       </c>
       <c r="J25" t="n">
-        <v>0.1359</v>
+        <v>0.1772</v>
       </c>
       <c r="K25" t="n">
-        <v>0.0004</v>
+        <v>0.0005</v>
       </c>
       <c r="L25" t="n">
-        <v>968.9</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="26">
@@ -1594,31 +1594,31 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>5.864</v>
+        <v>7.3846</v>
       </c>
       <c r="E26" t="n">
-        <v>0.1279</v>
+        <v>0.4183</v>
       </c>
       <c r="F26" t="n">
-        <v>4.1525</v>
+        <v>5.9345</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1226</v>
+        <v>0.313</v>
       </c>
       <c r="H26" t="n">
-        <v>0.7007</v>
+        <v>0.7772</v>
       </c>
       <c r="I26" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0003</v>
       </c>
       <c r="J26" t="n">
-        <v>0.1358</v>
+        <v>0.1761</v>
       </c>
       <c r="K26" t="n">
         <v>0.0003</v>
       </c>
       <c r="L26" t="n">
-        <v>968.9</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="27">
@@ -1638,31 +1638,31 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>41.2313</v>
+        <v>19.6401</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>41.2396</v>
+        <v>19.8536</v>
       </c>
       <c r="G27" t="n">
         <v>0</v>
       </c>
       <c r="H27" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>0.4023</v>
+        <v>0.2348</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>1381.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="28">
@@ -1682,31 +1682,31 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>23.0101</v>
+        <v>11.9216</v>
       </c>
       <c r="E28" t="n">
-        <v>0.0083</v>
+        <v>0.0211</v>
       </c>
       <c r="F28" t="n">
-        <v>22.1304</v>
+        <v>11.2831</v>
       </c>
       <c r="G28" t="n">
-        <v>0.0385</v>
+        <v>0.0387</v>
       </c>
       <c r="H28" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0.2239</v>
+        <v>0.1919</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L28" t="n">
-        <v>1381.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="29">
@@ -1726,31 +1726,31 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>5.6909</v>
+        <v>6.7292</v>
       </c>
       <c r="E29" t="n">
-        <v>0.007900000000000001</v>
+        <v>0.0167</v>
       </c>
       <c r="F29" t="n">
-        <v>3.8419</v>
+        <v>6.0678</v>
       </c>
       <c r="G29" t="n">
-        <v>0.08119999999999999</v>
+        <v>0.1836</v>
       </c>
       <c r="H29" t="n">
-        <v>0.698</v>
+        <v>0.765</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>0.1383</v>
+        <v>0.1787</v>
       </c>
       <c r="K29" t="n">
         <v>0.0001</v>
       </c>
       <c r="L29" t="n">
-        <v>1381.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="30">
@@ -1770,31 +1770,31 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5.9911</v>
+        <v>7.2717</v>
       </c>
       <c r="E30" t="n">
-        <v>0.1181</v>
+        <v>0.1836</v>
       </c>
       <c r="F30" t="n">
-        <v>4.6814</v>
+        <v>6.5486</v>
       </c>
       <c r="G30" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.1657</v>
       </c>
       <c r="H30" t="n">
-        <v>0.7201</v>
+        <v>0.7781</v>
       </c>
       <c r="I30" t="n">
-        <v>0.0009</v>
+        <v>0.0004</v>
       </c>
       <c r="J30" t="n">
-        <v>0.1356</v>
+        <v>0.1769</v>
       </c>
       <c r="K30" t="n">
         <v>0.0001</v>
       </c>
       <c r="L30" t="n">
-        <v>1381.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="31">
@@ -1814,31 +1814,31 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6.091</v>
+        <v>7.6659</v>
       </c>
       <c r="E31" t="n">
-        <v>0.0891</v>
+        <v>0.1268</v>
       </c>
       <c r="F31" t="n">
-        <v>4.3094</v>
+        <v>6.0513</v>
       </c>
       <c r="G31" t="n">
-        <v>0.08450000000000001</v>
+        <v>0.1345</v>
       </c>
       <c r="H31" t="n">
-        <v>0.7008</v>
+        <v>0.7772</v>
       </c>
       <c r="I31" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="J31" t="n">
-        <v>0.1359</v>
+        <v>0.1762</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L31" t="n">
-        <v>1381.5</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="32">
@@ -1858,31 +1858,31 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>41.2313</v>
+        <v>19.6401</v>
       </c>
       <c r="E32" t="n">
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>41.2396</v>
+        <v>19.8536</v>
       </c>
       <c r="G32" t="n">
         <v>0</v>
       </c>
       <c r="H32" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>0.4023</v>
+        <v>0.2348</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>1460.1</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="33">
@@ -1902,31 +1902,31 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>23.0146</v>
+        <v>11.9356</v>
       </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>22.1877</v>
+        <v>11.3174</v>
       </c>
       <c r="G33" t="n">
         <v>0</v>
       </c>
       <c r="H33" t="n">
-        <v>0.6742</v>
+        <v>0.765</v>
       </c>
       <c r="I33" t="n">
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>0.2239</v>
+        <v>0.1919</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>1460.1</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="34">
@@ -1946,31 +1946,31 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>5.6927</v>
+        <v>6.7343</v>
       </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>3.9037</v>
+        <v>6.2134</v>
       </c>
       <c r="G34" t="n">
         <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>0.698</v>
+        <v>0.765</v>
       </c>
       <c r="I34" t="n">
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0.1383</v>
+        <v>0.1788</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>1460.1</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="35">
@@ -1990,31 +1990,31 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>5.8519</v>
+        <v>7.1458</v>
       </c>
       <c r="E35" t="n">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>4.7714</v>
+        <v>6.5587</v>
       </c>
       <c r="G35" t="n">
         <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>0.7202</v>
+        <v>0.7782</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>0.1356</v>
+        <v>0.1769</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>1460.1</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="36">
@@ -2034,31 +2034,31 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>6.167</v>
+        <v>7.6674</v>
       </c>
       <c r="E36" t="n">
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>4.2981</v>
+        <v>6.1614</v>
       </c>
       <c r="G36" t="n">
         <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>0.7006</v>
+        <v>0.7772</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>0.1359</v>
+        <v>0.1762</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>1460.1</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="37">
@@ -2078,25 +2078,25 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>32.75</v>
+        <v>24.5955</v>
       </c>
       <c r="E37" t="n">
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>33.2705</v>
+        <v>24.8438</v>
       </c>
       <c r="G37" t="n">
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>0.3163</v>
+        <v>0.258</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -2122,28 +2122,28 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>24.5418</v>
+        <v>17.4034</v>
       </c>
       <c r="E38" t="n">
-        <v>0.1368</v>
+        <v>0.144</v>
       </c>
       <c r="F38" t="n">
-        <v>24.2989</v>
+        <v>17.2866</v>
       </c>
       <c r="G38" t="n">
-        <v>0.2627</v>
+        <v>0.1384</v>
       </c>
       <c r="H38" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>0.2192</v>
+        <v>0.2175</v>
       </c>
       <c r="K38" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0009</v>
       </c>
       <c r="L38" t="n">
         <v>50</v>
@@ -2166,28 +2166,28 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>8.230700000000001</v>
+        <v>9.8942</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3621</v>
+        <v>0.7315</v>
       </c>
       <c r="F39" t="n">
-        <v>6.6734</v>
+        <v>9.0288</v>
       </c>
       <c r="G39" t="n">
-        <v>0.2321</v>
+        <v>1.0437</v>
       </c>
       <c r="H39" t="n">
-        <v>0.674</v>
+        <v>0.7256</v>
       </c>
       <c r="I39" t="n">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0.1378</v>
+        <v>0.1883</v>
       </c>
       <c r="K39" t="n">
-        <v>0.0011</v>
+        <v>0.0024</v>
       </c>
       <c r="L39" t="n">
         <v>50</v>
@@ -2210,28 +2210,28 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8.2666</v>
+        <v>9.4886</v>
       </c>
       <c r="E40" t="n">
-        <v>0.4171</v>
+        <v>0.9439</v>
       </c>
       <c r="F40" t="n">
-        <v>7.2965</v>
+        <v>8.8569</v>
       </c>
       <c r="G40" t="n">
-        <v>0.4856</v>
+        <v>1.2554</v>
       </c>
       <c r="H40" t="n">
-        <v>0.6641</v>
+        <v>0.724</v>
       </c>
       <c r="I40" t="n">
-        <v>0.0204</v>
+        <v>0.0139</v>
       </c>
       <c r="J40" t="n">
-        <v>0.1407</v>
+        <v>0.1889</v>
       </c>
       <c r="K40" t="n">
-        <v>0.0021</v>
+        <v>0.0056</v>
       </c>
       <c r="L40" t="n">
         <v>50</v>
@@ -2254,28 +2254,28 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>8.1561</v>
+        <v>9.507</v>
       </c>
       <c r="E41" t="n">
-        <v>0.6168</v>
+        <v>1.0866</v>
       </c>
       <c r="F41" t="n">
-        <v>6.9676</v>
+        <v>8.879</v>
       </c>
       <c r="G41" t="n">
-        <v>0.721</v>
+        <v>1.5399</v>
       </c>
       <c r="H41" t="n">
-        <v>0.6697</v>
+        <v>0.7324000000000001</v>
       </c>
       <c r="I41" t="n">
-        <v>0.0031</v>
+        <v>0.0016</v>
       </c>
       <c r="J41" t="n">
-        <v>0.141</v>
+        <v>0.1872</v>
       </c>
       <c r="K41" t="n">
-        <v>0.0042</v>
+        <v>0.0037</v>
       </c>
       <c r="L41" t="n">
         <v>50</v>
@@ -2298,25 +2298,25 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>32.75</v>
+        <v>24.5955</v>
       </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>33.2705</v>
+        <v>24.8438</v>
       </c>
       <c r="G42" t="n">
         <v>0</v>
       </c>
       <c r="H42" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0.3163</v>
+        <v>0.258</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2342,28 +2342,28 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>24.4165</v>
+        <v>17.2835</v>
       </c>
       <c r="E43" t="n">
-        <v>0.1636</v>
+        <v>0.454</v>
       </c>
       <c r="F43" t="n">
-        <v>24.0793</v>
+        <v>17.0797</v>
       </c>
       <c r="G43" t="n">
-        <v>0.3834</v>
+        <v>0.555</v>
       </c>
       <c r="H43" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0.2186</v>
+        <v>0.2165</v>
       </c>
       <c r="K43" t="n">
-        <v>0.0007</v>
+        <v>0.0014</v>
       </c>
       <c r="L43" t="n">
         <v>100</v>
@@ -2386,28 +2386,28 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>7.5364</v>
+        <v>9.116899999999999</v>
       </c>
       <c r="E44" t="n">
-        <v>0.0951</v>
+        <v>0.3629</v>
       </c>
       <c r="F44" t="n">
-        <v>5.9528</v>
+        <v>7.9364</v>
       </c>
       <c r="G44" t="n">
-        <v>0.4314</v>
+        <v>0.7876</v>
       </c>
       <c r="H44" t="n">
-        <v>0.674</v>
+        <v>0.7256</v>
       </c>
       <c r="I44" t="n">
-        <v>0.0106</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0.1358</v>
+        <v>0.1857</v>
       </c>
       <c r="K44" t="n">
-        <v>0.0002</v>
+        <v>0.0011</v>
       </c>
       <c r="L44" t="n">
         <v>100</v>
@@ -2430,28 +2430,28 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>7.1606</v>
+        <v>8.0589</v>
       </c>
       <c r="E45" t="n">
-        <v>0.5702</v>
+        <v>0.7633</v>
       </c>
       <c r="F45" t="n">
-        <v>6.3048</v>
+        <v>7.3312</v>
       </c>
       <c r="G45" t="n">
-        <v>0.6885</v>
+        <v>1.0282</v>
       </c>
       <c r="H45" t="n">
-        <v>0.7017</v>
+        <v>0.742</v>
       </c>
       <c r="I45" t="n">
-        <v>0.0188</v>
+        <v>0.008</v>
       </c>
       <c r="J45" t="n">
-        <v>0.1364</v>
+        <v>0.183</v>
       </c>
       <c r="K45" t="n">
-        <v>0.002</v>
+        <v>0.0038</v>
       </c>
       <c r="L45" t="n">
         <v>100</v>
@@ -2474,28 +2474,28 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>6.9058</v>
+        <v>8.335599999999999</v>
       </c>
       <c r="E46" t="n">
-        <v>0.4821</v>
+        <v>0.6317</v>
       </c>
       <c r="F46" t="n">
-        <v>5.7473</v>
+        <v>7.4514</v>
       </c>
       <c r="G46" t="n">
-        <v>0.6072</v>
+        <v>0.6556</v>
       </c>
       <c r="H46" t="n">
-        <v>0.6808</v>
+        <v>0.7337</v>
       </c>
       <c r="I46" t="n">
-        <v>0.0067</v>
+        <v>0.002</v>
       </c>
       <c r="J46" t="n">
-        <v>0.1358</v>
+        <v>0.1838</v>
       </c>
       <c r="K46" t="n">
-        <v>0.0018</v>
+        <v>0.0011</v>
       </c>
       <c r="L46" t="n">
         <v>100</v>
@@ -2518,25 +2518,25 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>32.75</v>
+        <v>24.5955</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>33.2705</v>
+        <v>24.8438</v>
       </c>
       <c r="G47" t="n">
         <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>0.3163</v>
+        <v>0.258</v>
       </c>
       <c r="K47" t="n">
         <v>0</v>
@@ -2562,28 +2562,28 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>24.2811</v>
+        <v>17.0852</v>
       </c>
       <c r="E48" t="n">
-        <v>0.122</v>
+        <v>0.3436</v>
       </c>
       <c r="F48" t="n">
-        <v>23.9232</v>
+        <v>17.0461</v>
       </c>
       <c r="G48" t="n">
-        <v>0.1937</v>
+        <v>0.3572</v>
       </c>
       <c r="H48" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>0.2181</v>
+        <v>0.216</v>
       </c>
       <c r="K48" t="n">
-        <v>0.0003</v>
+        <v>0.0008</v>
       </c>
       <c r="L48" t="n">
         <v>200</v>
@@ -2606,28 +2606,28 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>7.3413</v>
+        <v>9.0243</v>
       </c>
       <c r="E49" t="n">
-        <v>0.1156</v>
+        <v>0.2496</v>
       </c>
       <c r="F49" t="n">
-        <v>5.6314</v>
+        <v>8.065899999999999</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1357</v>
+        <v>0.2851</v>
       </c>
       <c r="H49" t="n">
-        <v>0.6745</v>
+        <v>0.7256</v>
       </c>
       <c r="I49" t="n">
-        <v>0.0117</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>0.135</v>
+        <v>0.185</v>
       </c>
       <c r="K49" t="n">
-        <v>0.0003</v>
+        <v>0.0005</v>
       </c>
       <c r="L49" t="n">
         <v>200</v>
@@ -2650,28 +2650,28 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>6.5795</v>
+        <v>7.081</v>
       </c>
       <c r="E50" t="n">
-        <v>0.3681</v>
+        <v>0.6108</v>
       </c>
       <c r="F50" t="n">
-        <v>5.6836</v>
+        <v>6.5605</v>
       </c>
       <c r="G50" t="n">
-        <v>0.349</v>
+        <v>0.7006</v>
       </c>
       <c r="H50" t="n">
-        <v>0.7037</v>
+        <v>0.7463</v>
       </c>
       <c r="I50" t="n">
-        <v>0.0142</v>
+        <v>0.0045</v>
       </c>
       <c r="J50" t="n">
-        <v>0.134</v>
+        <v>0.1809</v>
       </c>
       <c r="K50" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0016</v>
       </c>
       <c r="L50" t="n">
         <v>200</v>
@@ -2694,28 +2694,28 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6.6186</v>
+        <v>8.059200000000001</v>
       </c>
       <c r="E51" t="n">
-        <v>0.1925</v>
+        <v>0.4936</v>
       </c>
       <c r="F51" t="n">
-        <v>5.2331</v>
+        <v>7.0731</v>
       </c>
       <c r="G51" t="n">
-        <v>0.357</v>
+        <v>0.2503</v>
       </c>
       <c r="H51" t="n">
-        <v>0.68</v>
+        <v>0.7339</v>
       </c>
       <c r="I51" t="n">
-        <v>0.0064</v>
+        <v>0.0019</v>
       </c>
       <c r="J51" t="n">
-        <v>0.1337</v>
+        <v>0.1823</v>
       </c>
       <c r="K51" t="n">
-        <v>0.0005</v>
+        <v>0.0009</v>
       </c>
       <c r="L51" t="n">
         <v>200</v>
@@ -2738,25 +2738,25 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>32.75</v>
+        <v>24.5955</v>
       </c>
       <c r="E52" t="n">
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>33.2705</v>
+        <v>24.8438</v>
       </c>
       <c r="G52" t="n">
         <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>0.3163</v>
+        <v>0.258</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
@@ -2782,28 +2782,28 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>24.3248</v>
+        <v>17.2465</v>
       </c>
       <c r="E53" t="n">
-        <v>0.0862</v>
+        <v>0.2458</v>
       </c>
       <c r="F53" t="n">
-        <v>23.9307</v>
+        <v>17.2793</v>
       </c>
       <c r="G53" t="n">
-        <v>0.1259</v>
+        <v>0.2793</v>
       </c>
       <c r="H53" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>0.2183</v>
+        <v>0.2165</v>
       </c>
       <c r="K53" t="n">
-        <v>0.0002</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="L53" t="n">
         <v>500</v>
@@ -2826,28 +2826,28 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>7.2675</v>
+        <v>9.028499999999999</v>
       </c>
       <c r="E54" t="n">
-        <v>0.0866</v>
+        <v>0.2377</v>
       </c>
       <c r="F54" t="n">
-        <v>5.2966</v>
+        <v>7.8955</v>
       </c>
       <c r="G54" t="n">
-        <v>0.1364</v>
+        <v>0.2119</v>
       </c>
       <c r="H54" t="n">
-        <v>0.6744</v>
+        <v>0.7256</v>
       </c>
       <c r="I54" t="n">
-        <v>0.0117</v>
+        <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>0.1348</v>
+        <v>0.185</v>
       </c>
       <c r="K54" t="n">
-        <v>0.0001</v>
+        <v>0.0004</v>
       </c>
       <c r="L54" t="n">
         <v>500</v>
@@ -2870,28 +2870,28 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>6.4085</v>
+        <v>7.3599</v>
       </c>
       <c r="E55" t="n">
-        <v>0.3408</v>
+        <v>0.6617</v>
       </c>
       <c r="F55" t="n">
-        <v>5.4261</v>
+        <v>6.4867</v>
       </c>
       <c r="G55" t="n">
-        <v>0.4091</v>
+        <v>0.925</v>
       </c>
       <c r="H55" t="n">
-        <v>0.7216</v>
+        <v>0.7524999999999999</v>
       </c>
       <c r="I55" t="n">
-        <v>0.014</v>
+        <v>0.003</v>
       </c>
       <c r="J55" t="n">
-        <v>0.1324</v>
+        <v>0.1783</v>
       </c>
       <c r="K55" t="n">
-        <v>0.0004</v>
+        <v>0.0007</v>
       </c>
       <c r="L55" t="n">
         <v>500</v>
@@ -2914,28 +2914,28 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>6.6139</v>
+        <v>8.2308</v>
       </c>
       <c r="E56" t="n">
-        <v>0.2072</v>
+        <v>0.3482</v>
       </c>
       <c r="F56" t="n">
-        <v>4.9984</v>
+        <v>7.1699</v>
       </c>
       <c r="G56" t="n">
-        <v>0.3213</v>
+        <v>0.4199</v>
       </c>
       <c r="H56" t="n">
-        <v>0.6862</v>
+        <v>0.7343</v>
       </c>
       <c r="I56" t="n">
-        <v>0.0024</v>
+        <v>0.0003</v>
       </c>
       <c r="J56" t="n">
-        <v>0.1333</v>
+        <v>0.1818</v>
       </c>
       <c r="K56" t="n">
-        <v>0.0001</v>
+        <v>0.0003</v>
       </c>
       <c r="L56" t="n">
         <v>500</v>
@@ -2958,31 +2958,31 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>32.75</v>
+        <v>24.5955</v>
       </c>
       <c r="E57" t="n">
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>33.2705</v>
+        <v>24.8438</v>
       </c>
       <c r="G57" t="n">
         <v>0</v>
       </c>
       <c r="H57" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>0.3163</v>
+        <v>0.258</v>
       </c>
       <c r="K57" t="n">
         <v>0</v>
       </c>
       <c r="L57" t="n">
-        <v>906.1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="58">
@@ -3002,31 +3002,31 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>24.2458</v>
+        <v>17.0312</v>
       </c>
       <c r="E58" t="n">
-        <v>0.062</v>
+        <v>0.1737</v>
       </c>
       <c r="F58" t="n">
-        <v>23.9217</v>
+        <v>17.1583</v>
       </c>
       <c r="G58" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.1933</v>
       </c>
       <c r="H58" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>0.2181</v>
+        <v>0.2161</v>
       </c>
       <c r="K58" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="L58" t="n">
-        <v>906.1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="59">
@@ -3046,31 +3046,31 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>7.1551</v>
+        <v>8.8302</v>
       </c>
       <c r="E59" t="n">
-        <v>0.0287</v>
+        <v>0.0806</v>
       </c>
       <c r="F59" t="n">
-        <v>5.3729</v>
+        <v>7.8699</v>
       </c>
       <c r="G59" t="n">
-        <v>0.1438</v>
+        <v>0.3549</v>
       </c>
       <c r="H59" t="n">
-        <v>0.6689000000000001</v>
+        <v>0.7256</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>0.1346</v>
+        <v>0.1846</v>
       </c>
       <c r="K59" t="n">
-        <v>0.0001</v>
+        <v>0.0004</v>
       </c>
       <c r="L59" t="n">
-        <v>906.1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="60">
@@ -3090,31 +3090,31 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>6.4129</v>
+        <v>6.7427</v>
       </c>
       <c r="E60" t="n">
-        <v>0.1601</v>
+        <v>0.5774</v>
       </c>
       <c r="F60" t="n">
-        <v>5.6095</v>
+        <v>6.1554</v>
       </c>
       <c r="G60" t="n">
-        <v>0.0934</v>
+        <v>0.2248</v>
       </c>
       <c r="H60" t="n">
-        <v>0.7386</v>
+        <v>0.7524</v>
       </c>
       <c r="I60" t="n">
-        <v>0.0011</v>
+        <v>0.0008</v>
       </c>
       <c r="J60" t="n">
-        <v>0.1319</v>
+        <v>0.1777</v>
       </c>
       <c r="K60" t="n">
         <v>0.0001</v>
       </c>
       <c r="L60" t="n">
-        <v>906.1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="61">
@@ -3134,31 +3134,31 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>6.7209</v>
+        <v>8.1249</v>
       </c>
       <c r="E61" t="n">
-        <v>0.1234</v>
+        <v>0.3479</v>
       </c>
       <c r="F61" t="n">
-        <v>5.0345</v>
+        <v>7.1549</v>
       </c>
       <c r="G61" t="n">
-        <v>0.154</v>
+        <v>0.3633</v>
       </c>
       <c r="H61" t="n">
-        <v>0.6889</v>
+        <v>0.7339</v>
       </c>
       <c r="I61" t="n">
-        <v>0.0007</v>
+        <v>0.0004</v>
       </c>
       <c r="J61" t="n">
-        <v>0.1332</v>
+        <v>0.1815</v>
       </c>
       <c r="K61" t="n">
-        <v>0.0001</v>
+        <v>0.0003</v>
       </c>
       <c r="L61" t="n">
-        <v>906.1</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="62">
@@ -3178,31 +3178,31 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>32.75</v>
+        <v>24.5955</v>
       </c>
       <c r="E62" t="n">
         <v>0</v>
       </c>
       <c r="F62" t="n">
-        <v>33.2705</v>
+        <v>24.8438</v>
       </c>
       <c r="G62" t="n">
         <v>0</v>
       </c>
       <c r="H62" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I62" t="n">
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>0.3163</v>
+        <v>0.258</v>
       </c>
       <c r="K62" t="n">
         <v>0</v>
       </c>
       <c r="L62" t="n">
-        <v>1190.4</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="63">
@@ -3222,31 +3222,31 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>24.2221</v>
+        <v>16.9614</v>
       </c>
       <c r="E63" t="n">
-        <v>0.0217</v>
+        <v>0.0609</v>
       </c>
       <c r="F63" t="n">
-        <v>23.8601</v>
+        <v>16.9819</v>
       </c>
       <c r="G63" t="n">
-        <v>0.0242</v>
+        <v>0.0677</v>
       </c>
       <c r="H63" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I63" t="n">
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>0.218</v>
+        <v>0.2159</v>
       </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L63" t="n">
-        <v>1190.4</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="64">
@@ -3266,31 +3266,31 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>7.1599</v>
+        <v>8.845800000000001</v>
       </c>
       <c r="E64" t="n">
-        <v>0.014</v>
+        <v>0.0439</v>
       </c>
       <c r="F64" t="n">
-        <v>5.3252</v>
+        <v>7.8751</v>
       </c>
       <c r="G64" t="n">
-        <v>0.0468</v>
+        <v>0.09959999999999999</v>
       </c>
       <c r="H64" t="n">
-        <v>0.6689000000000001</v>
+        <v>0.7256</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>0.1346</v>
+        <v>0.1845</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L64" t="n">
-        <v>1190.4</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="65">
@@ -3310,31 +3310,31 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>6.558</v>
+        <v>7.1546</v>
       </c>
       <c r="E65" t="n">
-        <v>0.1254</v>
+        <v>0.382</v>
       </c>
       <c r="F65" t="n">
-        <v>5.4898</v>
+        <v>6.1191</v>
       </c>
       <c r="G65" t="n">
-        <v>0.1076</v>
+        <v>0.3053</v>
       </c>
       <c r="H65" t="n">
-        <v>0.7389</v>
+        <v>0.7522</v>
       </c>
       <c r="I65" t="n">
         <v>0.0005</v>
       </c>
       <c r="J65" t="n">
-        <v>0.1319</v>
+        <v>0.1777</v>
       </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L65" t="n">
-        <v>1190.4</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="66">
@@ -3354,31 +3354,31 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>6.5876</v>
+        <v>7.9298</v>
       </c>
       <c r="E66" t="n">
-        <v>0.0354</v>
+        <v>0.1396</v>
       </c>
       <c r="F66" t="n">
-        <v>5.0661</v>
+        <v>7.2139</v>
       </c>
       <c r="G66" t="n">
-        <v>0.0551</v>
+        <v>0.1488</v>
       </c>
       <c r="H66" t="n">
-        <v>0.6891</v>
+        <v>0.734</v>
       </c>
       <c r="I66" t="n">
         <v>0.0001</v>
       </c>
       <c r="J66" t="n">
-        <v>0.1331</v>
+        <v>0.1814</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="L66" t="n">
-        <v>1190.4</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="67">
@@ -3398,31 +3398,31 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>32.75</v>
+        <v>24.5955</v>
       </c>
       <c r="E67" t="n">
         <v>0</v>
       </c>
       <c r="F67" t="n">
-        <v>33.2705</v>
+        <v>24.8438</v>
       </c>
       <c r="G67" t="n">
         <v>0</v>
       </c>
       <c r="H67" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I67" t="n">
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>0.3163</v>
+        <v>0.258</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
       </c>
       <c r="L67" t="n">
-        <v>1240.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="68">
@@ -3442,31 +3442,31 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>24.2151</v>
+        <v>16.9418</v>
       </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
       <c r="F68" t="n">
-        <v>23.8038</v>
+        <v>16.8242</v>
       </c>
       <c r="G68" t="n">
         <v>0</v>
       </c>
       <c r="H68" t="n">
-        <v>0.669</v>
+        <v>0.7256</v>
       </c>
       <c r="I68" t="n">
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>0.218</v>
+        <v>0.2158</v>
       </c>
       <c r="K68" t="n">
         <v>0</v>
       </c>
       <c r="L68" t="n">
-        <v>1240.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="69">
@@ -3486,31 +3486,31 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>7.1567</v>
+        <v>8.837899999999999</v>
       </c>
       <c r="E69" t="n">
         <v>0</v>
       </c>
       <c r="F69" t="n">
-        <v>5.3856</v>
+        <v>7.9324</v>
       </c>
       <c r="G69" t="n">
         <v>0</v>
       </c>
       <c r="H69" t="n">
-        <v>0.6689000000000001</v>
+        <v>0.7256</v>
       </c>
       <c r="I69" t="n">
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>0.1346</v>
+        <v>0.1845</v>
       </c>
       <c r="K69" t="n">
         <v>0</v>
       </c>
       <c r="L69" t="n">
-        <v>1240.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="70">
@@ -3530,31 +3530,31 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>6.5016</v>
+        <v>7.1646</v>
       </c>
       <c r="E70" t="n">
         <v>0</v>
       </c>
       <c r="F70" t="n">
-        <v>5.5625</v>
+        <v>6.2351</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
       </c>
       <c r="H70" t="n">
-        <v>0.739</v>
+        <v>0.7522</v>
       </c>
       <c r="I70" t="n">
         <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>0.1319</v>
+        <v>0.1778</v>
       </c>
       <c r="K70" t="n">
         <v>0</v>
       </c>
       <c r="L70" t="n">
-        <v>1240.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="71">
@@ -3574,31 +3574,31 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>6.5658</v>
+        <v>7.8853</v>
       </c>
       <c r="E71" t="n">
         <v>0</v>
       </c>
       <c r="F71" t="n">
-        <v>5.0274</v>
+        <v>7.0833</v>
       </c>
       <c r="G71" t="n">
         <v>0</v>
       </c>
       <c r="H71" t="n">
-        <v>0.6889</v>
+        <v>0.734</v>
       </c>
       <c r="I71" t="n">
         <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0.1331</v>
+        <v>0.1814</v>
       </c>
       <c r="K71" t="n">
         <v>0</v>
       </c>
       <c r="L71" t="n">
-        <v>1240.4</v>
+        <v>1600</v>
       </c>
     </row>
     <row r="72"/>
@@ -5366,25 +5366,25 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>6.1833</v>
+        <v>4.3006</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
       </c>
       <c r="G37" t="n">
-        <v>7.0398</v>
+        <v>4.0114</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>0.103</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
@@ -5412,28 +5412,28 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>6.0337</v>
+        <v>4.9468</v>
       </c>
       <c r="F38" t="n">
-        <v>0.4162</v>
+        <v>1.3692</v>
       </c>
       <c r="G38" t="n">
-        <v>5.8875</v>
+        <v>3.7464</v>
       </c>
       <c r="H38" t="n">
-        <v>0.4484</v>
+        <v>1.984</v>
       </c>
       <c r="I38" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J38" t="n">
         <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>0.1024</v>
+        <v>0.0906</v>
       </c>
       <c r="L38" t="n">
-        <v>0.0009</v>
+        <v>0.0016</v>
       </c>
     </row>
     <row r="39">
@@ -5458,28 +5458,28 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>7.2169</v>
+        <v>5.7993</v>
       </c>
       <c r="F39" t="n">
-        <v>1.403</v>
+        <v>1.9641</v>
       </c>
       <c r="G39" t="n">
-        <v>6.0792</v>
+        <v>5.0441</v>
       </c>
       <c r="H39" t="n">
-        <v>1.3222</v>
+        <v>2.4582</v>
       </c>
       <c r="I39" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>0.1045</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="L39" t="n">
-        <v>0.0023</v>
+        <v>0.0052</v>
       </c>
     </row>
     <row r="40">
@@ -5504,28 +5504,28 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>5.2298</v>
+        <v>5.5205</v>
       </c>
       <c r="F40" t="n">
-        <v>1.1611</v>
+        <v>1.6385</v>
       </c>
       <c r="G40" t="n">
-        <v>3.5517</v>
+        <v>5.177</v>
       </c>
       <c r="H40" t="n">
-        <v>1.2112</v>
+        <v>1.7582</v>
       </c>
       <c r="I40" t="n">
-        <v>0.7675999999999999</v>
+        <v>0.8347</v>
       </c>
       <c r="J40" t="n">
-        <v>0.011</v>
+        <v>0.03</v>
       </c>
       <c r="K40" t="n">
-        <v>0.1107</v>
+        <v>0.09959999999999999</v>
       </c>
       <c r="L40" t="n">
-        <v>0.0026</v>
+        <v>0.0067</v>
       </c>
     </row>
     <row r="41">
@@ -5550,28 +5550,28 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>6.0944</v>
+        <v>6.0504</v>
       </c>
       <c r="F41" t="n">
-        <v>0.6462</v>
+        <v>2.6295</v>
       </c>
       <c r="G41" t="n">
-        <v>5.161</v>
+        <v>5.8314</v>
       </c>
       <c r="H41" t="n">
-        <v>1.0908</v>
+        <v>3.1944</v>
       </c>
       <c r="I41" t="n">
-        <v>0.8155</v>
+        <v>0.871</v>
       </c>
       <c r="J41" t="n">
-        <v>0.0023</v>
+        <v>0.0048</v>
       </c>
       <c r="K41" t="n">
-        <v>0.1036</v>
+        <v>0.09660000000000001</v>
       </c>
       <c r="L41" t="n">
-        <v>0.0017</v>
+        <v>0.0109</v>
       </c>
     </row>
     <row r="42">
@@ -5596,25 +5596,25 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>6.1833</v>
+        <v>4.3006</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
       </c>
       <c r="G42" t="n">
-        <v>7.0398</v>
+        <v>4.0114</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J42" t="n">
         <v>0</v>
       </c>
       <c r="K42" t="n">
-        <v>0.103</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L42" t="n">
         <v>0</v>
@@ -5642,28 +5642,28 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>5.7244</v>
+        <v>4.882</v>
       </c>
       <c r="F43" t="n">
-        <v>0.2755</v>
+        <v>0.6591</v>
       </c>
       <c r="G43" t="n">
-        <v>5.5024</v>
+        <v>3.4533</v>
       </c>
       <c r="H43" t="n">
-        <v>0.5425</v>
+        <v>1.395</v>
       </c>
       <c r="I43" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>0.1018</v>
+        <v>0.0902</v>
       </c>
       <c r="L43" t="n">
-        <v>0.0003</v>
+        <v>0.0007</v>
       </c>
     </row>
     <row r="44">
@@ -5688,28 +5688,28 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>5.6942</v>
+        <v>5.2224</v>
       </c>
       <c r="F44" t="n">
-        <v>0.9481000000000001</v>
+        <v>1.0161</v>
       </c>
       <c r="G44" t="n">
-        <v>5.3301</v>
+        <v>4.4699</v>
       </c>
       <c r="H44" t="n">
-        <v>1.0174</v>
+        <v>0.9077</v>
       </c>
       <c r="I44" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>0.1019</v>
+        <v>0.0911</v>
       </c>
       <c r="L44" t="n">
-        <v>0.0012</v>
+        <v>0.0021</v>
       </c>
     </row>
     <row r="45">
@@ -5734,28 +5734,28 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>5.0566</v>
+        <v>4.7682</v>
       </c>
       <c r="F45" t="n">
-        <v>0.6182</v>
+        <v>0.367</v>
       </c>
       <c r="G45" t="n">
-        <v>4.3824</v>
+        <v>4.7215</v>
       </c>
       <c r="H45" t="n">
-        <v>1.0198</v>
+        <v>0.9804</v>
       </c>
       <c r="I45" t="n">
-        <v>0.7936</v>
+        <v>0.8466</v>
       </c>
       <c r="J45" t="n">
-        <v>0.0114</v>
+        <v>0.0163</v>
       </c>
       <c r="K45" t="n">
-        <v>0.1046</v>
+        <v>0.0968</v>
       </c>
       <c r="L45" t="n">
-        <v>0.0021</v>
+        <v>0.0045</v>
       </c>
     </row>
     <row r="46">
@@ -5780,28 +5780,28 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>5.3563</v>
+        <v>5.1458</v>
       </c>
       <c r="F46" t="n">
-        <v>1.2421</v>
+        <v>1.1491</v>
       </c>
       <c r="G46" t="n">
-        <v>4.8101</v>
+        <v>4.579</v>
       </c>
       <c r="H46" t="n">
-        <v>0.7255</v>
+        <v>0.5964</v>
       </c>
       <c r="I46" t="n">
-        <v>0.8165</v>
+        <v>0.8737</v>
       </c>
       <c r="J46" t="n">
-        <v>0.0033</v>
+        <v>0.0045</v>
       </c>
       <c r="K46" t="n">
-        <v>0.1015</v>
+        <v>0.09130000000000001</v>
       </c>
       <c r="L46" t="n">
-        <v>0.0009</v>
+        <v>0.0025</v>
       </c>
     </row>
     <row r="47">
@@ -5826,25 +5826,25 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>6.1833</v>
+        <v>4.3006</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
       </c>
       <c r="G47" t="n">
-        <v>7.0398</v>
+        <v>4.0114</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>0.103</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L47" t="n">
         <v>0</v>
@@ -5872,28 +5872,28 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>5.4872</v>
+        <v>4.9351</v>
       </c>
       <c r="F48" t="n">
-        <v>0.1421</v>
+        <v>0.421</v>
       </c>
       <c r="G48" t="n">
-        <v>5.7932</v>
+        <v>3.8428</v>
       </c>
       <c r="H48" t="n">
-        <v>0.4716</v>
+        <v>1.2635</v>
       </c>
       <c r="I48" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>0.1015</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L48" t="n">
-        <v>0.0002</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="49">
@@ -5918,28 +5918,28 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>4.907</v>
+        <v>4.5526</v>
       </c>
       <c r="F49" t="n">
-        <v>0.3262</v>
+        <v>0.5573</v>
       </c>
       <c r="G49" t="n">
-        <v>5.0839</v>
+        <v>3.711</v>
       </c>
       <c r="H49" t="n">
-        <v>0.6334</v>
+        <v>0.8686</v>
       </c>
       <c r="I49" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
       </c>
       <c r="K49" t="n">
-        <v>0.1009</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="L49" t="n">
-        <v>0.0004</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="50">
@@ -5964,28 +5964,28 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>5.2771</v>
+        <v>4.3689</v>
       </c>
       <c r="F50" t="n">
-        <v>1.022</v>
+        <v>0.6234</v>
       </c>
       <c r="G50" t="n">
-        <v>4.3415</v>
+        <v>4.6293</v>
       </c>
       <c r="H50" t="n">
-        <v>0.7148</v>
+        <v>0.6137</v>
       </c>
       <c r="I50" t="n">
-        <v>0.8119</v>
+        <v>0.8655</v>
       </c>
       <c r="J50" t="n">
-        <v>0.0039</v>
+        <v>0.0072</v>
       </c>
       <c r="K50" t="n">
-        <v>0.1021</v>
+        <v>0.0911</v>
       </c>
       <c r="L50" t="n">
-        <v>0.0014</v>
+        <v>0.0013</v>
       </c>
     </row>
     <row r="51">
@@ -6010,28 +6010,28 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>5.231</v>
+        <v>4.297</v>
       </c>
       <c r="F51" t="n">
-        <v>0.3499</v>
+        <v>0.4528</v>
       </c>
       <c r="G51" t="n">
-        <v>4.8331</v>
+        <v>3.7293</v>
       </c>
       <c r="H51" t="n">
-        <v>0.7903</v>
+        <v>0.5834</v>
       </c>
       <c r="I51" t="n">
-        <v>0.8179999999999999</v>
+        <v>0.8735000000000001</v>
       </c>
       <c r="J51" t="n">
-        <v>0.0029</v>
+        <v>0.0017</v>
       </c>
       <c r="K51" t="n">
-        <v>0.1006</v>
+        <v>0.0892</v>
       </c>
       <c r="L51" t="n">
-        <v>0.0003</v>
+        <v>0.0005999999999999999</v>
       </c>
     </row>
     <row r="52">
@@ -6056,25 +6056,25 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>6.1833</v>
+        <v>4.3006</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>7.0398</v>
+        <v>4.0114</v>
       </c>
       <c r="H52" t="n">
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J52" t="n">
         <v>0</v>
       </c>
       <c r="K52" t="n">
-        <v>0.103</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L52" t="n">
         <v>0</v>
@@ -6102,28 +6102,28 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>5.4791</v>
+        <v>4.7741</v>
       </c>
       <c r="F53" t="n">
-        <v>0.0837</v>
+        <v>0.2009</v>
       </c>
       <c r="G53" t="n">
-        <v>5.6713</v>
+        <v>3.1241</v>
       </c>
       <c r="H53" t="n">
-        <v>0.2017</v>
+        <v>0.4255</v>
       </c>
       <c r="I53" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J53" t="n">
         <v>0</v>
       </c>
       <c r="K53" t="n">
-        <v>0.1015</v>
+        <v>0.0901</v>
       </c>
       <c r="L53" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
     </row>
     <row r="54">
@@ -6148,28 +6148,28 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>4.9358</v>
+        <v>4.2439</v>
       </c>
       <c r="F54" t="n">
-        <v>0.2721</v>
+        <v>0.3853</v>
       </c>
       <c r="G54" t="n">
-        <v>4.4246</v>
+        <v>3.4448</v>
       </c>
       <c r="H54" t="n">
-        <v>0.5204</v>
+        <v>0.3754</v>
       </c>
       <c r="I54" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J54" t="n">
         <v>0</v>
       </c>
       <c r="K54" t="n">
-        <v>0.1009</v>
+        <v>0.0888</v>
       </c>
       <c r="L54" t="n">
-        <v>0.0003</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="55">
@@ -6194,28 +6194,28 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>4.8538</v>
+        <v>4.6702</v>
       </c>
       <c r="F55" t="n">
-        <v>0.8648</v>
+        <v>0.916</v>
       </c>
       <c r="G55" t="n">
-        <v>5.2703</v>
+        <v>3.5407</v>
       </c>
       <c r="H55" t="n">
-        <v>0.8696</v>
+        <v>0.6286</v>
       </c>
       <c r="I55" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8697</v>
       </c>
       <c r="J55" t="n">
-        <v>0.0039</v>
+        <v>0.0009</v>
       </c>
       <c r="K55" t="n">
-        <v>0.1024</v>
+        <v>0.0891</v>
       </c>
       <c r="L55" t="n">
-        <v>0.0011</v>
+        <v>0.0004</v>
       </c>
     </row>
     <row r="56">
@@ -6240,25 +6240,25 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>5.4163</v>
+        <v>4.1834</v>
       </c>
       <c r="F56" t="n">
-        <v>0.3489</v>
+        <v>0.4227</v>
       </c>
       <c r="G56" t="n">
-        <v>4.546</v>
+        <v>3.8058</v>
       </c>
       <c r="H56" t="n">
-        <v>0.406</v>
+        <v>0.6843</v>
       </c>
       <c r="I56" t="n">
-        <v>0.8154</v>
+        <v>0.8733</v>
       </c>
       <c r="J56" t="n">
-        <v>0.0026</v>
+        <v>0.001</v>
       </c>
       <c r="K56" t="n">
-        <v>0.1006</v>
+        <v>0.0887</v>
       </c>
       <c r="L56" t="n">
         <v>0.0004</v>
@@ -6286,25 +6286,25 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>6.1833</v>
+        <v>4.3006</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
       </c>
       <c r="G57" t="n">
-        <v>7.0398</v>
+        <v>4.0114</v>
       </c>
       <c r="H57" t="n">
         <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J57" t="n">
         <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>0.103</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L57" t="n">
         <v>0</v>
@@ -6332,28 +6332,28 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>5.4187</v>
+        <v>4.8462</v>
       </c>
       <c r="F58" t="n">
-        <v>0.0244</v>
+        <v>0.1073</v>
       </c>
       <c r="G58" t="n">
-        <v>5.8391</v>
+        <v>3.3098</v>
       </c>
       <c r="H58" t="n">
-        <v>0.2161</v>
+        <v>0.3167</v>
       </c>
       <c r="I58" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>0.1014</v>
+        <v>0.0901</v>
       </c>
       <c r="L58" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
     </row>
     <row r="59">
@@ -6378,28 +6378,28 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>4.7729</v>
+        <v>4.4407</v>
       </c>
       <c r="F59" t="n">
-        <v>0.1025</v>
+        <v>0.1899</v>
       </c>
       <c r="G59" t="n">
-        <v>4.9542</v>
+        <v>3.5113</v>
       </c>
       <c r="H59" t="n">
-        <v>0.3217</v>
+        <v>0.5691000000000001</v>
       </c>
       <c r="I59" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J59" t="n">
         <v>0</v>
       </c>
       <c r="K59" t="n">
-        <v>0.1007</v>
+        <v>0.089</v>
       </c>
       <c r="L59" t="n">
-        <v>0.0001</v>
+        <v>0.0003</v>
       </c>
     </row>
     <row r="60">
@@ -6424,28 +6424,28 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>5.3447</v>
+        <v>3.9733</v>
       </c>
       <c r="F60" t="n">
-        <v>0.1389</v>
+        <v>0.5144</v>
       </c>
       <c r="G60" t="n">
-        <v>5.0576</v>
+        <v>3.5325</v>
       </c>
       <c r="H60" t="n">
-        <v>0.3663</v>
+        <v>0.4631</v>
       </c>
       <c r="I60" t="n">
-        <v>0.8191000000000001</v>
+        <v>0.8715000000000001</v>
       </c>
       <c r="J60" t="n">
-        <v>0.0024</v>
+        <v>0.0019</v>
       </c>
       <c r="K60" t="n">
-        <v>0.1005</v>
+        <v>0.08989999999999999</v>
       </c>
       <c r="L60" t="n">
-        <v>0.0003</v>
+        <v>0.0005</v>
       </c>
     </row>
     <row r="61">
@@ -6470,25 +6470,25 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>5.1214</v>
+        <v>4.3694</v>
       </c>
       <c r="F61" t="n">
-        <v>0.4776</v>
+        <v>0.1593</v>
       </c>
       <c r="G61" t="n">
-        <v>4.6877</v>
+        <v>3.2739</v>
       </c>
       <c r="H61" t="n">
-        <v>0.4904</v>
+        <v>0.2644</v>
       </c>
       <c r="I61" t="n">
-        <v>0.8164</v>
+        <v>0.8741</v>
       </c>
       <c r="J61" t="n">
-        <v>0.0018</v>
+        <v>0.001</v>
       </c>
       <c r="K61" t="n">
-        <v>0.1004</v>
+        <v>0.0887</v>
       </c>
       <c r="L61" t="n">
         <v>0.0002</v>
@@ -6512,29 +6512,29 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>6.1833</v>
+        <v>4.3006</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
       </c>
       <c r="G62" t="n">
-        <v>7.0398</v>
+        <v>4.0114</v>
       </c>
       <c r="H62" t="n">
         <v>0</v>
       </c>
       <c r="I62" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J62" t="n">
         <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>0.103</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L62" t="n">
         <v>0</v>
@@ -6558,29 +6558,29 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>5.4359</v>
+        <v>4.9317</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
       </c>
       <c r="G63" t="n">
-        <v>5.8593</v>
+        <v>3.5194</v>
       </c>
       <c r="H63" t="n">
         <v>0</v>
       </c>
       <c r="I63" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J63" t="n">
         <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>0.1014</v>
+        <v>0.0902</v>
       </c>
       <c r="L63" t="n">
         <v>0</v>
@@ -6604,29 +6604,29 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>4.7929</v>
+        <v>4.6377</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>4.3717</v>
+        <v>3.9672</v>
       </c>
       <c r="H64" t="n">
         <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J64" t="n">
         <v>0</v>
       </c>
       <c r="K64" t="n">
-        <v>0.1007</v>
+        <v>0.0893</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
@@ -6650,29 +6650,29 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>5.5891</v>
+        <v>4.4801</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
       </c>
       <c r="G65" t="n">
-        <v>3.9525</v>
+        <v>3.5505</v>
       </c>
       <c r="H65" t="n">
         <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>0.8184</v>
+        <v>0.8728</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>0.1008</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L65" t="n">
         <v>0</v>
@@ -6696,29 +6696,29 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>5.218</v>
+        <v>4.492</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
       </c>
       <c r="G66" t="n">
-        <v>4.9011</v>
+        <v>3.8365</v>
       </c>
       <c r="H66" t="n">
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.8742</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
       </c>
       <c r="K66" t="n">
-        <v>0.1004</v>
+        <v>0.089</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -6742,29 +6742,29 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>6.1833</v>
+        <v>4.3006</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
       </c>
       <c r="G67" t="n">
-        <v>7.0398</v>
+        <v>4.0114</v>
       </c>
       <c r="H67" t="n">
         <v>0</v>
       </c>
       <c r="I67" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
       </c>
       <c r="K67" t="n">
-        <v>0.103</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L67" t="n">
         <v>0</v>
@@ -6788,29 +6788,29 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>5.4359</v>
+        <v>4.9317</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
       </c>
       <c r="G68" t="n">
-        <v>5.8593</v>
+        <v>3.5194</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
       </c>
       <c r="I68" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
       </c>
       <c r="K68" t="n">
-        <v>0.1014</v>
+        <v>0.0902</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
@@ -6834,29 +6834,29 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>4.7929</v>
+        <v>4.6377</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
       </c>
       <c r="G69" t="n">
-        <v>4.3717</v>
+        <v>3.9672</v>
       </c>
       <c r="H69" t="n">
         <v>0</v>
       </c>
       <c r="I69" t="n">
-        <v>0.8178</v>
+        <v>0.8756</v>
       </c>
       <c r="J69" t="n">
         <v>0</v>
       </c>
       <c r="K69" t="n">
-        <v>0.1007</v>
+        <v>0.0893</v>
       </c>
       <c r="L69" t="n">
         <v>0</v>
@@ -6880,29 +6880,29 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>5.5891</v>
+        <v>4.4801</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
       </c>
       <c r="G70" t="n">
-        <v>3.9525</v>
+        <v>3.5505</v>
       </c>
       <c r="H70" t="n">
         <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>0.8184</v>
+        <v>0.8728</v>
       </c>
       <c r="J70" t="n">
         <v>0</v>
       </c>
       <c r="K70" t="n">
-        <v>0.1008</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L70" t="n">
         <v>0</v>
@@ -6926,29 +6926,29 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>1481 (Full)</t>
+          <t>1276 (Full)</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>5.218</v>
+        <v>4.492</v>
       </c>
       <c r="F71" t="n">
         <v>0</v>
       </c>
       <c r="G71" t="n">
-        <v>4.9011</v>
+        <v>3.8365</v>
       </c>
       <c r="H71" t="n">
         <v>0</v>
       </c>
       <c r="I71" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.8742</v>
       </c>
       <c r="J71" t="n">
         <v>0</v>
       </c>
       <c r="K71" t="n">
-        <v>0.1004</v>
+        <v>0.089</v>
       </c>
       <c r="L71" t="n">
         <v>0</v>

</xml_diff>